<commit_message>
Record deployed recruitment UI verification in review workbook
</commit_message>
<xml_diff>
--- a/outputs/recruit-connect-20261023/Rize Recruit - Traceability Matrix - Connections review.xlsx
+++ b/outputs/recruit-connect-20261023/Rize Recruit - Traceability Matrix - Connections review.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tested and status" sheetId="1" r:id="R35a102cc2dcf4edc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yet to be tested" sheetId="2" r:id="R4ea5344da771435a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tested and status" sheetId="1" r:id="R5b59d6621a2f4164"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yet to be tested" sheetId="2" r:id="R594f1a30996b4ab9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1311,7 +1311,7 @@
       </x:c>
       <x:c r="H3" s="15" t="str">
         <x:v>PARTIAL — code deployed / calendar setup required
-Added official Google/Microsoft SDK panel free/busy checks, expiring single-use candidate booking, browser timezone selection and a fresh conflict check before booking. Native calendar time changes create an interview audit trail. Automated booking and reschedule tests pass. Rize IT: configure OAuth applications, tenant consent and panel-calendar permissions; each organiser connects their calendar. Payobook/Rize: complete a controlled Google and Outlook booking/sync test. No live provider consent or availability is claimed.</x:v>
+Added official Google/Microsoft SDK panel free/busy checks, expiring single-use candidate booking, browser timezone selection and a fresh conflict check before booking. Native calendar time changes create an interview audit trail. Automated booking and reschedule tests pass. Chrome verified the booking form preserves the existing Asia/Calcutta timezone alias. Rize IT: configure OAuth applications, tenant consent and panel-calendar permissions; each organiser connects their calendar. Payobook/Rize: complete a controlled Google and Outlook booking/sync test. No live provider consent or availability is claimed.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="166" customHeight="1">
@@ -1413,7 +1413,7 @@
       </x:c>
       <x:c r="H7" s="15" t="str">
         <x:v>PARTIAL — access setup required
-Added Hiring only profile: unrelated sidebar/search entries and the Access directory are hidden; server access to that directory and its role catalogue is refused. Applied to the two demo TA logins. Recruiter handles candidates; Talent lead additionally manages hiring setup, country rules and retention. Rize administrator: assign this profile with the appropriate hiring role to real TA users, remove independent HR/payroll/admin grants, and complete negative-access tests. This profile does not revoke separately granted permissions.</x:v>
+Added Hiring only profile: unrelated sidebar/search entries and the Access directory are hidden; server access to that directory and its role catalogue is refused. Applied to the two demo TA logins. Recruiter handles candidates; Talent lead additionally manages hiring setup, country rules and retention. Rize administrator: assign this profile with the appropriate hiring role to real TA users, remove independent HR/payroll/admin grants, and complete negative-access tests. This profile does not revoke separately granted permissions. Deployed Chrome/API checks passed for both demo roles; Recruiter sees hiring rules read-only and cannot load connection settings.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="124" customHeight="1">
@@ -2233,7 +2233,7 @@
     </x:row>
     <x:row r="45" ht="160" customHeight="1">
       <x:c r="H45" s="19" t="str">
-        <x:v>Release dd3aaaacf (implementation ae2ae077c). pb_hiring 19.0.2.12.0; pb_hub 19.0.1.12.2. Deployed: payobook, payobook_template, p0clone, rize. 29 Odoo regression tests and 6 CV-service tests passed; deployed demo-role/API and public-token checks passed. Chrome asset load passed; full Hiring wizard UI check pending permission to switch the existing Komal session. External provider activation/live tests pending.</x:v>
+        <x:v>Release e9a60a7d7 (implementation ae2ae077c). pb_hiring 19.0.2.12.1; pb_hub 19.0.1.12.2. Deployed: payobook, payobook_template, p0clone, rize. 30 Odoo regression tests and 6 CV-service tests passed. Deployed demo-role/API and public-token checks passed. Chrome verified setup guides, keyboard navigation, native forms, timezone defaults and role restrictions. External provider activation/live tests remain pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15.75" customHeight="1">
@@ -3274,7 +3274,7 @@
         <x:v>175</x:v>
       </x:c>
       <x:c r="J2" s="21" t="str">
-        <x:v>NOT CLIENT-TESTED — Added explicit TA Lead and Head of HR fallback with dated absence handling; self-approval is blocked and no org-chart fallback is assumed. Automated routing tests pass. Rize TA Lead/administrator: configure the named approvers per country, then test normal approval, lead absence, requester-is-lead and cover reversion. Client test-result cells remain unchanged.</x:v>
+        <x:v>NOT CLIENT-TESTED — Added explicit TA Lead and Head of HR fallback with dated absence handling; self-approval is blocked and no org-chart fallback is assumed. Automated routing tests pass. Fixed access to existing rule forms; Chrome verified the named approver and absence-date fields. Rize TA Lead/administrator: configure the named approvers per country, then test normal approval, lead absence, requester-is-lead and cover reversion. Client test-result cells remain unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="166" customHeight="1">
@@ -3824,7 +3824,7 @@
     </x:row>
     <x:row r="30" ht="160" customHeight="1">
       <x:c r="J30" s="19" t="str">
-        <x:v>Release dd3aaaacf (implementation ae2ae077c). pb_hiring 19.0.2.12.0; pb_hub 19.0.1.12.2. Deployed: payobook, payobook_template, p0clone, rize. 29 Odoo regression tests and 6 CV-service tests passed; deployed demo-role/API and public-token checks passed. Chrome asset load passed; full Hiring wizard UI check pending permission to switch the existing Komal session. External provider activation/live tests pending.</x:v>
+        <x:v>Release e9a60a7d7 (implementation ae2ae077c). pb_hiring 19.0.2.12.1; pb_hub 19.0.1.12.2. Deployed: payobook, payobook_template, p0clone, rize. 30 Odoo regression tests and 6 CV-service tests passed. Deployed demo-role/API and public-token checks passed. Chrome verified setup guides, keyboard navigation, native forms, timezone defaults and role restrictions. External provider activation/live tests remain pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15.75" customHeight="1">

</xml_diff>

<commit_message>
Update recruitment review with DocuSign deployment and CV-only sizing
</commit_message>
<xml_diff>
--- a/outputs/recruit-connect-20261023/Rize Recruit - Traceability Matrix - Connections review.xlsx
+++ b/outputs/recruit-connect-20261023/Rize Recruit - Traceability Matrix - Connections review.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tested and status" sheetId="1" r:id="R5b59d6621a2f4164"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yet to be tested" sheetId="2" r:id="R594f1a30996b4ab9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tested and status" sheetId="1" r:id="Rfb00ffc4311347ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yet to be tested" sheetId="2" r:id="R7dd1cd8224d04331"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1686,7 +1686,7 @@
 Added explicit company/country/effective-date offer profiles using Payobook payroll formulas for employer-cost estimates. Required inputs cannot silently default to zero; monthly, annual and first-year one-time costs are separate. Pay changes invalidate estimates. Automated calculation tests pass. Rize HR/Finance: approve the payroll configuration, input/output mappings, defaults/rates, country letter and counter-signatory; administrator enters these in Country offer setup. No statutory rates were invented and estimates do not post payroll.</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="138" customHeight="1">
+    <x:row r="18" ht="152" customHeight="1">
       <x:c r="A18" s="2" t="s">
         <x:v>83</x:v>
       </x:c>
@@ -1709,8 +1709,8 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="H18" s="15" t="str">
-        <x:v>PARTIAL — Documenso POC coded / activation pending
-Added Documenso draft preparation, signer/field review, sending, cancellation/restart, authenticated completion verification and signed-PDF filing. Active signatures lock offer terms; verified completion invokes existing signed-offer workflow once. Automated signing-state tests pass with mocked provider responses. Required: service hosting, HTTPS, PostgreSQL, verified SMTP, signing certificate, team API key and webhook secret. Complete a controlled live signing/archive round trip before acceptance. This is a proof of concept, not a live-certified signing service.</x:v>
+        <x:v>PARTIAL — DocuSign coded / account activation pending
+Replaced new-offer signing with DocuSign: company-scoped encrypted JWT credentials, draft creation/recovery, reviewed signer and required-signature checks, send/void/restart, HMAC callbacks, API-verified completion and signed-PDF filing including the completion certificate. Twelve DocuSign regression tests pass with mocked provider responses. Required: DocuSign eSignature API entitlement, integration/user/account IDs, RSA key, sender consent and account Connect HMAC key. Run a controlled live signing/archive test before acceptance. No self-hosted signing server is required; existing legacy envelopes retain their original provider.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="110" customHeight="1">
@@ -1767,7 +1767,7 @@
 Fixed agency attribution and late-feedback counts. New direct careers applications get Careers page; internal additions/imports get Manual entry / import unless a specific source is supplied. Existing unknown sources are preserved rather than guessed. Recruiter: correct historical sources from evidence and choose specific sources for imports. Time-to-fill uses opened_on to filled_on (role opening to final signature after this fix), not request agreement; agency joining time is labelled separately.</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="110" customHeight="1">
+    <x:row r="21" ht="96" customHeight="1">
       <x:c r="A21" s="2" t="s">
         <x:v>96</x:v>
       </x:c>
@@ -1789,7 +1789,7 @@
       </x:c>
       <x:c r="H21" s="15" t="str">
         <x:v>PARTIAL — code deployed / setup and provider test
-Country employer-cost calculation, explicit letter/signatory setup and Documenso signing integration are now coded; see REC-025/026. Rize HR/Finance must approve country formulas, rates, letters and signers. Administrator configures country profiles; service hosting/credentials and a live signing/archive test remain pending. Manual configuration is acceptable but is not marked as completed.</x:v>
+Country employer-cost calculation, explicit letter/signatory setup and DocuSign signing integration are coded; see REC-025/026. HR/Finance approves country formulas, rates, letters and signers. Administrator configures profiles and DocuSign API account/consent/keys. A controlled live signing/archive test remains pending. No custom signing server is needed.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="124" customHeight="1">
@@ -2233,7 +2233,7 @@
     </x:row>
     <x:row r="45" ht="160" customHeight="1">
       <x:c r="H45" s="19" t="str">
-        <x:v>Release e9a60a7d7 (implementation ae2ae077c). pb_hiring 19.0.2.12.1; pb_hub 19.0.1.12.2. Deployed: payobook, payobook_template, p0clone, rize. 30 Odoo regression tests and 6 CV-service tests passed. Deployed demo-role/API and public-token checks passed. Chrome verified setup guides, keyboard navigation, native forms, timezone defaults and role restrictions. External provider activation/live tests remain pending.</x:v>
+        <x:v>Release f7cd70ae0 (DocuSign). pb_hiring 19.0.2.13.0; pb_hub 19.0.1.12.2. Deployed: payobook, payobook_template, p0clone, rize. 42 recruitment regression tests passed, including 12 DocuSign tests. Deployed Chrome setup/offer controls and role/API checks passed. Six earlier CV-service tests passed. DocuSign demo account creation, credentials, consent and live signing/archive test remain pending; CV hosting is unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15.75" customHeight="1">
@@ -3824,7 +3824,7 @@
     </x:row>
     <x:row r="30" ht="160" customHeight="1">
       <x:c r="J30" s="19" t="str">
-        <x:v>Release e9a60a7d7 (implementation ae2ae077c). pb_hiring 19.0.2.12.1; pb_hub 19.0.1.12.2. Deployed: payobook, payobook_template, p0clone, rize. 30 Odoo regression tests and 6 CV-service tests passed. Deployed demo-role/API and public-token checks passed. Chrome verified setup guides, keyboard navigation, native forms, timezone defaults and role restrictions. External provider activation/live tests remain pending.</x:v>
+        <x:v>Release f7cd70ae0 (DocuSign). pb_hiring 19.0.2.13.0; pb_hub 19.0.1.12.2. Deployed: payobook, payobook_template, p0clone, rize. 42 recruitment regression tests passed, including 12 DocuSign tests. Deployed Chrome setup/offer controls and role/API checks passed. Six earlier CV-service tests passed. DocuSign demo account creation, credentials, consent and live signing/archive test remain pending; CV hosting is unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15.75" customHeight="1">

</xml_diff>